<commit_message>
Update scheme 2 compute parameters
</commit_message>
<xml_diff>
--- a/estore_schemes/2/params.xlsx
+++ b/estore_schemes/2/params.xlsx
@@ -63657,7 +63657,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -63672,7 +63672,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>300</v>
+        <v>3600</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -63687,7 +63687,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.05</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -63702,7 +63702,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -63734,7 +63734,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -63893,7 +63893,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -63908,7 +63908,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -63923,7 +63923,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -63938,7 +63938,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>

</xml_diff>